<commit_message>
feat(F-NAR-019): ATOM-EMO.LEX.001-02 Raphaël et le gâteau à la vanille
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.LEX.001-02.xlsx
+++ b/stories/arbres/ATOM-EMO.LEX.001-02.xlsx
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>La vanille monte l'escalier. Raphaël descend. Il voit le gâteau aux fraises. Il dit sa joie. Il tend une fraise.</t>
+          <t>La pluie tapote la vitre. Raphaël connaît la cuisine. Sur le métal, un éclat de moule luit. Il veut le gâteau, maintenant. Je suis content, dit-il. Le moule penche. Poitrine trop vite. Sourire parti. Papa s'accroupit. Deuxième ruse : gâteau trop chaud, fraise qui glisse. Il refuse de foncer. Il tend la fraise. Merci vécu. Un éclat de moule tient sur le métal.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La vanille monte l'escalier, goutte à goutte. Elle sent le chaud et le doux. Dehors, la pluie tapote les carreaux. La gouttière chante un petit air. Dans la maison, papa et maman sont en bas. Raphaël est en haut, près de la rampe. Le bois de la rampe est lisse et tiède. Ses chaussettes glissent un tout petit peu. Raphaël, tu sens ça ? Ça sent le gâteau ! Viens voir. Le gâteau est prêt. En ce moment, Raphaël descend les marches. Une marche. Encore une marche. La cuisine est claire et tiède. Des gouttes courent sur la vitre. Sur la table, un gâteau rond attend. Des fraises rouges brillent dessus. Raphaël s'approche tout doucement. Tu veux le regarder de près ? Oui, maman. Il pose les mains sur la table. Le bois de la table est un peu collant. Ça sent la vanille tout fort. Parce que le gâteau est là, ses joues deviennent chaudes. Son ventre est léger, tout léger. Un sourire arrive tout seul. Je suis content. C'est de la joie. La joie, on peut la dire. Tu as nommé ta joie. Bravo, Raphaël. Raphaël regarde les fraises. Il en prend une, tout doucement. On peut partager ? Oui. On partage la joie aussi. Raphaël tend la fraise vers papa. Merci. Tu m'invites. C'est gentil. Papa prend un petit bout. Raphaël prend un petit bout. C'est sucré. C'est doux. Je suis content. Tu as encore de la joie ? Oui, papa. Maman se penche aussi. Maman, un bout pour toi. Merci, mon grand. Ils goûtent ensemble, tout près de la table. La pluie continue, plus douce.</t>
+          <t>La pluie tapote la vitre de la cuisine. Ça chante, papa. Tu l'entends, la pluie ? Oui, papa. Raphaël connaît cette cuisine, ses bruits, son air chaud. Tu la connais, cette pièce ? Oui, maman. Un détail paraît nouveau, près du four. Sur le métal, un éclat de moule luit. Il brille, maman. Tu le vois, sur le métal ? Oui, un petit point. Le four le touche. L'air sent le chaud et le sucré. Ça sent le gâteau ! Le gâteau à la vanille est dans le moule. Des fraises rouges brillent dessus. Elles sont rouges ! Tu les vois, les fraises ? Oui, papa. Le bois de la table est un peu collant. Il colle aux doigts. Il est tiède, Raphaël ? Un peu, maman. Le moule pèse un peu, sur la table. Il est lourd. Tu le sens, le poids ? Oui, papa. En ce moment, Raphaël avance vers le moule. Je veux le gâteau, maintenant ! Tout de suite ? Oui, papa. Ses joues deviennent chaudes. Son ventre est léger, très léger. Un sourire arrive, tout seul. Je suis content. Tes joues sont chaudes, Raphaël ? Oui, maman. Il tire le moule vers lui, trop vite. Le moule penche d'un coup. Le gâteau reste coincé, au fond. Ça fait un bruit sec. Oh. Raphaël reste surpris, les mains ouvertes. Sa poitrine va trop vite. Le sourire de Raphaël disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois le moule, Raphaël ? Oui, papa. Tes mains sont chaudes, Raphaël ? Un peu, maman. L'éclat de moule tremble, puis tient.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La vanille monte l'escalier, goutte à goutte. Elle sent le chaud et le doux. Dehors, la pluie tapote les carreaux. La gouttière chante un petit air. Dans la maison, papa et maman sont en bas. Raphaël est en haut, près de la rampe. Le bois de la rampe est lisse et tiède. Ses chaussettes glissent un tout petit peu. Raphaël, tu sens ça ? Ça sent le gâteau ! Viens voir. Le gâteau est prêt. En ce moment, Raphaël descend les marches. Une marche. Encore une marche. La cuisine est claire et tiède. Des gouttes courent sur la vitre. Sur la table, un gâteau rond attend. Des fraises rouges brillent dessus. Raphaël s'approche tout doucement. Tu veux le regarder de près ? Oui, maman. Il pose les mains sur la table. Le bois de la table est un peu collant. Ça sent la vanille tout fort. Parce que le gâteau est là, ses joues deviennent chaudes. Son ventre est léger, tout léger. Un sourire arrive tout seul. Je suis content. C'est de la joie. La joie, on peut la dire. Tu as nommé ta joie. Bravo, Raphaël. Raphaël regarde les fraises. Il en prend une, tout doucement. On peut partager ? Oui. On partage la joie aussi. Raphaël tend la fraise vers papa. Merci. Tu m'invites. C'est gentil. Papa prend un petit bout. Raphaël prend un petit bout. C'est sucré. C'est doux. Je suis content. Tu as encore de la joie ? Oui, papa. Maman se penche aussi. Maman, un bout pour toi. Merci, mon grand. Ils goûtent ensemble, tout près de la table. La pluie continue, plus douce.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La pluie tapote la vitre de la cuisine. Ça chante, papa. Tu l'entends, la pluie ? Oui, papa. Raphaël connaît cette cuisine, ses bruits, son air chaud. Tu la connais, cette pièce ? Oui, maman. Un détail paraît nouveau, près du four. Sur le métal, un &lt;emphasis level="moderate"&gt;éclat de moule&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, sur le métal ? Oui, un petit point. Le four le touche. L'air sent le chaud et le sucré. Ça sent le gâteau ! Le gâteau à la vanille est dans le moule. Des fraises rouges brillent dessus. Elles sont rouges ! Tu les vois, les fraises ? Oui, papa. Le bois de la table est un peu collant. Il colle aux doigts. Il est tiède, Raphaël ? Un peu, maman. Le moule pèse un peu, sur la table. Il est lourd. Tu le sens, le poids ? Oui, papa. En ce moment, Raphaël avance vers le moule. Je veux le gâteau, maintenant ! Tout de suite ? Oui, papa. Ses joues deviennent chaudes. Son ventre est léger, très léger. Un sourire arrive, tout seul. Je suis content. Tes joues sont chaudes, Raphaël ? Oui, maman. Il tire le moule vers lui, trop vite. Le moule penche d'un coup. Le gâteau reste coincé, au fond. Ça fait un bruit sec. Oh. Raphaël reste surpris, les mains ouvertes. Sa poitrine va trop vite. Le sourire de Raphaël disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois le moule, Raphaël ? Oui, papa. Tes mains sont chaudes, Raphaël ? Un peu, maman. L'éclat de moule tremble, puis tient.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Ava est dans la cuisine. Maman sort le gâteau. Ça sent la vanille. Papa s'assoit près de la table. Ava voit les fraises rouges. Parce que le gâteau est là, Ava sent ses joues chaudes. Son ventre est léger. Un sourire arrive. Ava dit : je suis &lt;emphasis&gt;content&lt;/emphasis&gt;e. Maman dit : c'est de la joie. Être content, c'est bien. Parce qu'elle a de la joie, Ava veut partager. Elle tend une fraise. Elle dit : on peut partager. Papa prend un petit bout. Ava prend un petit bout. Ils sourient ensemble. Ava dit encore : je suis contente. La joie est là, dans la cuisine. Maman sourit aussi. [pause]</t>
+          <t>La pluie tapote la vitre de la cuisine. Ça chante, papa. Tu l'entends, la pluie ? Oui, papa. Raphaël connaît cette cuisine, ses bruits, son air chaud. Tu la connais, cette pièce ? Oui, maman. Un détail paraît nouveau, près du four. Sur le métal, un &lt;emphasis&gt;éclat de moule&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, sur le métal ? Oui, un petit point. Le four le touche. L'air sent le chaud et le sucré. Ça sent le gâteau ! Le gâteau à la vanille est dans le moule. Des fraises rouges brillent dessus. Elles sont rouges ! Tu les vois, les fraises ? Oui, papa. Le bois de la table est un peu collant. Il colle aux doigts. Il est tiède, Raphaël ? Un peu, maman. Le moule pèse un peu, sur la table. Il est lourd. Tu le sens, le poids ? Oui, papa. En ce moment, Raphaël avance vers le moule. Je veux le gâteau, maintenant ! Tout de suite ? Oui, papa. Ses joues deviennent chaudes. Son ventre est léger, très léger. Un sourire arrive, tout seul. Je suis content. Tes joues sont chaudes, Raphaël ? Oui, maman. Il tire le moule vers lui, trop vite. Le moule penche d'un coup. Le gâteau reste coincé, au fond. Ça fait un bruit sec. Oh. Raphaël reste surpris, les mains ouvertes. Sa poitrine va trop vite. Le sourire de Raphaël disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois le moule, Raphaël ? Oui, papa. Tes mains sont chaudes, Raphaël ? Un peu, maman. L'éclat de moule tremble, puis tient. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>content</t>
+          <t>éclat de moule</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,60 +1321,68 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=joie puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_le_gateau_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La vanille monte l'escalier, goutte à goutte.
-narrateur|Elle sent le chaud et le doux.
-narrateur|Dehors, la pluie tapote les carreaux.
-narrateur|La gouttière chante un petit air.
-narrateur|Dans la maison, papa et maman sont en bas.
-narrateur|Raphaël est en haut, près de la rampe.
-narrateur|Le bois de la rampe est lisse et tiède.
-narrateur|Ses chaussettes glissent un tout petit peu.
-papa|Raphaël, tu sens ça ?
+          <t>narrateur|La pluie tapote la vitre de la cuisine.
+enfant-m|Ça chante, papa.
+papa|Tu l'entends, la pluie ?
+enfant-m|Oui, papa.
+narrateur|Raphaël connaît cette cuisine, ses bruits, son air chaud.
+maman|Tu la connais, cette pièce ?
+enfant-m|Oui, maman.
+narrateur|Un détail paraît nouveau, près du four.
+narrateur|Sur le métal, un éclat de moule luit.
+enfant-m|Il brille, maman.
+maman|Tu le vois, sur le métal ?
+enfant-m|Oui, un petit point.
+papa|Le four le touche.
+narrateur|L'air sent le chaud et le sucré.
 enfant-m|Ça sent le gâteau !
-maman|Viens voir.
-maman|Le gâteau est prêt.
-narrateur|En ce moment, Raphaël descend les marches.
-narrateur|Une marche. Encore une marche.
-narrateur|La cuisine est claire et tiède.
-narrateur|Des gouttes courent sur la vitre.
-narrateur|Sur la table, un gâteau rond attend.
+maman|Le gâteau à la vanille est dans le moule.
 narrateur|Des fraises rouges brillent dessus.
-narrateur|Raphaël s'approche tout doucement.
-maman|Tu veux le regarder de près ?
+enfant-m|Elles sont rouges !
+papa|Tu les vois, les fraises ?
+enfant-m|Oui, papa.
+narrateur|Le bois de la table est un peu collant.
+enfant-m|Il colle aux doigts.
+maman|Il est tiède, Raphaël ?
+enfant-m|Un peu, maman.
+narrateur|Le moule pèse un peu, sur la table.
+enfant-m|Il est lourd.
+papa|Tu le sens, le poids ?
+enfant-m|Oui, papa.
+narrateur|En ce moment, Raphaël avance vers le moule.
+enfant-m|Je veux le gâteau, maintenant !
+papa|Tout de suite ?
+enfant-m|Oui, papa.
+narrateur|Ses joues deviennent chaudes.
+narrateur|Son ventre est léger, très léger.
+narrateur|Un sourire arrive, tout seul.
+enfant-m|Je suis content.
+maman|Tes joues sont chaudes, Raphaël ?
 enfant-m|Oui, maman.
-narrateur|Il pose les mains sur la table.
-narrateur|Le bois de la table est un peu collant.
-narrateur|Ça sent la vanille tout fort.
-narrateur|Parce que le gâteau est là, ses joues deviennent chaudes.
-narrateur|Son ventre est léger, tout léger.
-narrateur|Un sourire arrive tout seul.
-enfant-m|Je suis content.
-maman|C'est de la joie.
-maman|La joie, on peut la dire.
-papa|Tu as nommé ta joie.
-papa|Bravo, Raphaël.
-narrateur|Raphaël regarde les fraises.
-narrateur|Il en prend une, tout doucement.
-enfant-m|On peut partager ?
-maman|Oui.
-maman|On partage la joie aussi.
-narrateur|Raphaël tend la fraise vers papa.
-papa|Merci.
-papa|Tu m'invites. C'est gentil.
-narrateur|Papa prend un petit bout.
-narrateur|Raphaël prend un petit bout.
-narrateur|C'est sucré. C'est doux.
-enfant-m|Je suis content.
-papa|Tu as encore de la joie ?
+narrateur|Il tire le moule vers lui, trop vite.
+narrateur|Le moule penche d'un coup.
+narrateur|Le gâteau reste coincé, au fond.
+narrateur|Ça fait un bruit sec.
+enfant-m|Oh.
+narrateur|Raphaël reste surpris, les mains ouvertes.
+narrateur|Sa poitrine va trop vite.
+narrateur|Le sourire de Raphaël disparaît.
+narrateur|Dans sa poitrine, ça se bouscule.
+narrateur|L'envie et l'inquiétude se heurtent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois le moule, Raphaël ?
 enfant-m|Oui, papa.
-narrateur|Maman se penche aussi.
-enfant-m|Maman, un bout pour toi.
-maman|Merci, mon grand.
-narrateur|Ils goûtent ensemble, tout près de la table.
-narrateur|La pluie continue, plus douce.</t>
+maman|Tes mains sont chaudes, Raphaël ?
+enfant-m|Un peu, maman.
+narrateur|L'éclat de moule tremble, puis tient.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1411,12 +1419,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Raphaël sourit. Que dit-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;&lt;emphasis level="moderate"&gt;Raphaël&lt;/emphasis&gt; sourit. Que dit-il ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Ava sourit. Que dit-elle ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;&lt;emphasis&gt;Raphaël&lt;/emphasis&gt; sourit. Que dit-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1441,7 +1449,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Ava sent de la joie. Que dit-elle ?</t>
+          <t>Raphaël sent de la joie. Que dit-il ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1479,7 +1487,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1490,7 +1498,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1505,34 +1513,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Raphaël</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1547,22 +1559,23 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=raphael_sourit_que_dit_il; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Raphaël sourit. Que dit-il ?</t>
+          <t>narrateur|Raphaël sourit.
+narrateur|Que dit-il ?</t>
         </is>
       </c>
     </row>
@@ -1589,17 +1602,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Raphaël a encore le bout de fraise. Il mâche tout doucement. C'est de la joie. Oui. Tu es content. Et tu as partagé. Tu as fini ton petit bout ? Oui. Raphaël essuie un peu de sucre au coin de la bouche. La vanille est encore dans l'air.</t>
+          <t>Raphaël veut le gâteau, tout de suite. Je le prends, maintenant ! Le moule reste un peu penché. Les mots se bousculent dans sa bouche. Trop vite. Raphaël avance les mains, trop vite. Puis il s'arrête. Il referme la bouche. Personne ne parle. Il observe le moule, un instant. Il écoute la cuisine, près du four. Il est coincé. Tu restes un peu, Raphaël ? Oui, papa. Papa reste à la même hauteur. Le métal est tiède, sous les doigts. Il pique un peu. Raphaël reprend le bord du moule, sans se presser. Tu le vois, le moule ? Oui, papa. Il tient, Raphaël ? Oui, maman. Le ventre de Raphaël se desserre. Les épaules se relèvent un peu. On reste près du moule ? Oui. La pluie tapote la vitre ? Oui, maman. Une fraise attend sur le dessus. Je la prends. Tu la poses, Raphaël ? Pas tout de suite. Le gâteau a un dessus un peu doré. Il est doré ! Tes genoux sont au chaud ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Raphaël a encore le bout de fraise. Il mâche tout doucement. C'est de la joie. Oui. Tu es content. Et tu as partagé. Tu as fini ton petit bout ? Oui. Raphaël essuie un peu de sucre au coin de la bouche. La vanille est encore dans l'air.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël veut le gâteau, tout de suite. Je le prends, maintenant ! Le &lt;emphasis level="moderate"&gt;moule&lt;/emphasis&gt; reste un peu penché. Les mots se bousculent dans sa bouche. Trop vite. Raphaël avance les mains, trop vite. Puis il s'arrête. Il referme la bouche. Personne ne parle. Il observe le moule, un instant. Il écoute la cuisine, près du four. Il est coincé. Tu restes un peu, Raphaël ? Oui, papa. Papa reste à la même hauteur. Le métal est tiède, sous les doigts. Il pique un peu. Raphaël reprend le bord du moule, sans se presser. Tu le vois, le moule ? Oui, papa. Il tient, Raphaël ? Oui, maman. Le ventre de Raphaël se desserre. Les épaules se relèvent un peu. On reste près du moule ? Oui. La pluie tapote la vitre ? Oui, maman. Une fraise attend sur le dessus. Je la prends. Tu la poses, Raphaël ? Pas tout de suite. Le gâteau a un dessus un peu doré. Il est doré ! Tes genoux sont au chaud ? Un peu, maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Ava a nommé sa joie. Elle a partagé avec papa et maman. Être &lt;emphasis&gt;content&lt;/emphasis&gt;, c'est bien. [pause]</t>
+          <t>Raphaël veut le gâteau, tout de suite. Je le prends, maintenant ! Le &lt;emphasis&gt;moule&lt;/emphasis&gt; reste un peu penché. Les mots se bousculent dans sa bouche. Trop vite. Raphaël avance les mains, trop vite. Puis il s'arrête. Il referme la bouche. Personne ne parle. Il observe le moule, un instant. Il écoute la cuisine, près du four. Il est coincé. Tu restes un peu, Raphaël ? Oui, papa. Papa reste à la même hauteur. Le métal est tiède, sous les doigts. Il pique un peu. Raphaël reprend le bord du moule, sans se presser. Tu le vois, le moule ? Oui, papa. Il tient, Raphaël ? Oui, maman. Le ventre de Raphaël se desserre. Les épaules se relèvent un peu. On reste près du moule ? Oui. La pluie tapote la vitre ? Oui, maman. Une fraise attend sur le dessus. Je la prends. Tu la poses, Raphaël ? Pas tout de suite. Le gâteau a un dessus un peu doré. Il est doré ! Tes genoux sont au chaud ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1657,7 +1670,7 @@
         <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1680,7 +1693,7 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>content</t>
+          <t>moule</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
@@ -1694,16 +1707,16 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1728,20 +1741,47 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer_sans_leçon; emotion=retenue puis joie_discrète; intensite=1; destinataire=enfant; sous_texte=il_s_arrete_le_moule_tient; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Raphaël a encore le bout de fraise.
-narrateur|Il mâche tout doucement.
-enfant-m|C'est de la joie.
-maman|Oui. Tu es content.
-maman|Et tu as partagé.
-papa|Tu as fini ton petit bout ?
+          <t>narrateur|Raphaël veut le gâteau, tout de suite.
+enfant-m|Je le prends, maintenant !
+narrateur|Le moule reste un peu penché.
+narrateur|Les mots se bousculent dans sa bouche.
+enfant-m|Trop vite.
+narrateur|Raphaël avance les mains, trop vite.
+narrateur|Puis il s'arrête.
+narrateur|Il referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Il observe le moule, un instant.
+narrateur|Il écoute la cuisine, près du four.
+enfant-m|Il est coincé.
+papa|Tu restes un peu, Raphaël ?
+enfant-m|Oui, papa.
+narrateur|Papa reste à la même hauteur.
+maman|Le métal est tiède, sous les doigts.
+enfant-m|Il pique un peu.
+narrateur|Raphaël reprend le bord du moule, sans se presser.
+papa|Tu le vois, le moule ?
+enfant-m|Oui, papa.
+maman|Il tient, Raphaël ?
+enfant-m|Oui, maman.
+narrateur|Le ventre de Raphaël se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|On reste près du moule ?
 enfant-m|Oui.
-narrateur|Raphaël essuie un peu de sucre au coin de la bouche.
-narrateur|La vanille est encore dans l'air.</t>
+maman|La pluie tapote la vitre ?
+enfant-m|Oui, maman.
+narrateur|Une fraise attend sur le dessus.
+enfant-m|Je la prends.
+papa|Tu la poses, Raphaël ?
+enfant-m|Pas tout de suite.
+narrateur|Le gâteau a un dessus un peu doré.
+enfant-m|Il est doré !
+maman|Tes genoux sont au chaud ?
+enfant-m|Un peu, maman.</t>
         </is>
       </c>
     </row>
@@ -1768,17 +1808,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Raphaël essuie ses mains sur la serviette. La cuisine sent encore le gâteau. On reste un peu à table ? Oui, maman. Tu as bien invité. Raphaël pose les pieds par terre. La pluie fait un bruit tout petit. Je suis content. La joie est là, avec nous. Ils restent près du gâteau, sans se presser.</t>
+          <t>Maman pousse le moule près de Raphaël. Le métal est un peu brûlant. Le gâteau, maintenant ! Raphaël approche la main, trop vite. La chaleur pique sa paume. Il est trop chaud ! Il retire la main d'un coup. Une fraise glisse du dessus. Elle glisse ! La fraise roule vers le bois de la table. Raphaël avance les mains, trop vite. Puis il s'arrête net. Raphaël refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le moule, un instant. Il écoute la cuisine, près du four. Sur le métal, un éclat de moule luit. Là, sur le métal. Raphaël attend, les mains ouvertes. On prend la fraise ? Oui, papa. La fraise sent le sucre, un peu tiède. Raphaël la tend vers papa. Merci, Raphaël. Papa prend un petit bout. Raphaël prend un petit bout. C'est sucré. Le sucre colle un peu, Raphaël ? Un peu. Tu vois le point, Raphaël ? Oui, papa. Le gâteau tient, dans le moule. On le garde. Un peu de pluie passe sur la vitre. Elle tapote. On reste ici, Raphaël ? Oui.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Raphaël essuie ses mains sur la serviette. La cuisine sent encore le gâteau. On reste un peu à table ? Oui, maman. Tu as bien invité. Raphaël pose les pieds par terre. La pluie fait un bruit tout petit. Je suis content. La joie est là, avec nous. Ils restent près du gâteau, sans se presser.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman pousse le moule près de Raphaël. Le métal est un peu brûlant. Le gâteau, maintenant ! Raphaël approche la main, trop vite. La chaleur pique sa paume. Il est trop chaud ! Il retire la main d'un coup. Une fraise glisse du dessus. Elle glisse ! La fraise roule vers le bois de la table. Raphaël avance les mains, trop vite. Puis il s'arrête net. Raphaël refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le moule, un instant. Il écoute la cuisine, près du four. Sur le métal, un &lt;emphasis level="moderate"&gt;éclat de moule&lt;/emphasis&gt; luit. Là, sur le métal. Raphaël attend, les mains ouvertes. On prend la fraise ? Oui, papa. La fraise sent le sucre, un peu tiède. Raphaël la tend vers papa. Merci, Raphaël. Papa prend un petit bout. Raphaël prend un petit bout. C'est sucré. Le sucre colle un peu, Raphaël ? Un peu. Tu vois le point, Raphaël ? Oui, papa. Le gâteau tient, dans le moule. On le garde. Un peu de pluie passe sur la vitre. Elle tapote. On reste ici, Raphaël ? Oui.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Ava essuie ses &lt;emphasis&gt;main&lt;/emphasis&gt;s. La cuisine sent encore bon. Maman lui prend la main. [pause]</t>
+          <t>Maman pousse le moule près de Raphaël. Le métal est un peu brûlant. Le gâteau, maintenant ! Raphaël approche la main, trop vite. La chaleur pique sa paume. Il est trop chaud ! Il retire la main d'un coup. Une fraise glisse du dessus. Elle glisse ! La fraise roule vers le bois de la table. Raphaël avance les mains, trop vite. Puis il s'arrête net. Raphaël refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le moule, un instant. Il écoute la cuisine, près du four. Sur le métal, un &lt;emphasis&gt;éclat de moule&lt;/emphasis&gt; luit. Là, sur le métal. Raphaël attend, les mains ouvertes. On prend la fraise ? Oui, papa. La fraise sent le sucre, un peu tiède. Raphaël la tend vers papa. Merci, Raphaël. Papa prend un petit bout. Raphaël prend un petit bout. C'est sucré. Le sucre colle un peu, Raphaël ? Un peu. Tu vois le point, Raphaël ? Oui, papa. Le gâteau tient, dans le moule. On le garde. Un peu de pluie passe sur la vitre. Elle tapote. On reste ici, Raphaël ? Oui. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1825,7 +1865,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1833,10 +1873,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.18</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1859,30 +1899,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de moule</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1891,10 +1931,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1905,19 +1945,56 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=gateau_trop_chaud_fraise_glisse_il_refuse_de_foncer; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Raphaël essuie ses mains sur la serviette.
-narrateur|La cuisine sent encore le gâteau.
-maman|On reste un peu à table ?
-enfant-m|Oui, maman.
-papa|Tu as bien invité.
-narrateur|Raphaël pose les pieds par terre.
-narrateur|La pluie fait un bruit tout petit.
-enfant-m|Je suis content.
-maman|La joie est là, avec nous.
-narrateur|Ils restent près du gâteau, sans se presser.</t>
+          <t>narrateur|Maman pousse le moule près de Raphaël.
+narrateur|Le métal est un peu brûlant.
+enfant-m|Le gâteau, maintenant !
+narrateur|Raphaël approche la main, trop vite.
+narrateur|La chaleur pique sa paume.
+enfant-m|Il est trop chaud !
+narrateur|Il retire la main d'un coup.
+narrateur|Une fraise glisse du dessus.
+enfant-m|Elle glisse !
+narrateur|La fraise roule vers le bois de la table.
+narrateur|Raphaël avance les mains, trop vite.
+narrateur|Puis il s'arrête net.
+narrateur|Raphaël refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Il observe le moule, un instant.
+narrateur|Il écoute la cuisine, près du four.
+narrateur|Sur le métal, un éclat de moule luit.
+enfant-m|Là, sur le métal.
+narrateur|Raphaël attend, les mains ouvertes.
+papa|On prend la fraise ?
+enfant-m|Oui, papa.
+narrateur|La fraise sent le sucre, un peu tiède.
+narrateur|Raphaël la tend vers papa.
+papa|Merci, Raphaël.
+narrateur|Papa prend un petit bout.
+narrateur|Raphaël prend un petit bout.
+enfant-m|C'est sucré.
+maman|Le sucre colle un peu, Raphaël ?
+enfant-m|Un peu.
+papa|Tu vois le point, Raphaël ?
+enfant-m|Oui, papa.
+narrateur|Le gâteau tient, dans le moule.
+enfant-m|On le garde.
+maman|Un peu de pluie passe sur la vitre.
+enfant-m|Elle tapote.
+papa|On reste ici, Raphaël ?
+enfant-m|Oui.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>pluie</t>
         </is>
       </c>
     </row>
@@ -1944,17 +2021,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis content. On a partagé la fraise. Bravo, Raphaël.</t>
+          <t>Ils restent près du moule. Maman essuie un peu de sucre. Le moule a penché, papa. Tu l'as vu, toi ? Oui, près du gâteau. On est bien, ici. Raphaël tapote le métal du doigt. Il a une trace de sucre. Tu la vois, la trace ? Oui, maman. Maman, un bout pour toi. Maman prend un petit bout. Le gâteau est resté, Raphaël. Oui, dans le moule. Ça sent la vanille, un peu tiède. Et le sucre, maman. Oui, dans l'air. La pluie tapote, Raphaël ? Oui, papa. Le moule reste près de la table. Un éclat de moule tient sur le métal.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis content. On a partagé la fraise. Bravo, Raphaël.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près du moule. Maman essuie un peu de sucre. Le moule a penché, papa. Tu l'as vu, toi ? Oui, près du gâteau. On est bien, ici. Raphaël tapote le métal du doigt. Il a une trace de sucre. Tu la vois, la trace ? Oui, maman. Maman, un bout pour toi. Maman prend un petit bout. Le gâteau est resté, Raphaël. Oui, dans le moule. Ça sent la vanille, un peu tiède. Et le sucre, maman. Oui, dans l'air. La pluie tapote, Raphaël ? Oui, papa. Le moule reste près de la table. Un &lt;emphasis level="moderate"&gt;éclat de moule&lt;/emphasis&gt; tient sur le métal.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près du moule. Maman essuie un peu de sucre. Le moule a penché, papa. Tu l'as vu, toi ? Oui, près du gâteau. On est bien, ici. Raphaël tapote le métal du doigt. Il a une trace de sucre. Tu la vois, la trace ? Oui, maman. Maman, un bout pour toi. Maman prend un petit bout. Le gâteau est resté, Raphaël. Oui, dans le moule. Ça sent la vanille, un peu tiède. Et le sucre, maman. Oui, dans l'air. La pluie tapote, Raphaël ? Oui, papa. Le moule reste près de la table. Un &lt;emphasis&gt;éclat de moule&lt;/emphasis&gt; tient sur le métal.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2001,7 +2078,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2009,10 +2086,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2021,12 +2098,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2035,17 +2112,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de moule</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2054,11 +2135,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2067,26 +2148,53 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_metal; tempo=très posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai dit : je suis content.
-enfant-m|On a partagé la fraise.
-papa|Bravo, Raphaël.</t>
+          <t>narrateur|Ils restent près du moule.
+narrateur|Maman essuie un peu de sucre.
+enfant-m|Le moule a penché, papa.
+papa|Tu l'as vu, toi ?
+enfant-m|Oui, près du gâteau.
+maman|On est bien, ici.
+narrateur|Raphaël tapote le métal du doigt.
+enfant-m|Il a une trace de sucre.
+maman|Tu la vois, la trace ?
+enfant-m|Oui, maman.
+enfant-m|Maman, un bout pour toi.
+narrateur|Maman prend un petit bout.
+papa|Le gâteau est resté, Raphaël.
+enfant-m|Oui, dans le moule.
+narrateur|Ça sent la vanille, un peu tiède.
+enfant-m|Et le sucre, maman.
+maman|Oui, dans l'air.
+papa|La pluie tapote, Raphaël ?
+enfant-m|Oui, papa.
+narrateur|Le moule reste près de la table.
+narrateur|Un éclat de moule tient sur le métal.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>pluie</t>
         </is>
       </c>
     </row>
@@ -2107,7 +2215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2157,6 +2265,13 @@
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>